<commit_message>
feat: Implement "My Assignments" tab in the audit window for auditors to fetch tasks, upload BRDs, and monitor live execution from a server.
</commit_message>
<xml_diff>
--- a/performance_dashboard/assets/template_test_cases.xlsx
+++ b/performance_dashboard/assets/template_test_cases.xlsx
@@ -658,46 +658,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Test Case ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Component</v>
+      </c>
+      <c r="C1" t="str">
         <v>Test Case Name</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Pre-requisites</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Test Steps</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>N-Points</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Iteration1</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Iteration2</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Iteration3</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Iteration4</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Iteration5</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Average</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Notes</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Baseline</v>
       </c>
     </row>
@@ -706,24 +709,24 @@
         <v>P02</v>
       </c>
       <c r="B2" t="str">
+        <v>OOBE</v>
+      </c>
+      <c r="C2" t="str">
         <v>Wake-up time from suspend - home</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v xml:space="preserve">wifi OFF, </v>
       </c>
-      <c r="D2" t="str" xml:space="preserve">
+      <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Register the device to given account.
  2. Device should be without ads, all the three books in home page should be with cover image
  3. Put the device in screen saver for 2.30 minutes(suspend).
  4. Press the power button and start the timer then stop the timer when the home page is settled.
  5. Repeat the above step for all the 5 iterations</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>10</v>
       </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
       <c r="G2" t="str">
         <v/>
       </c>
@@ -743,6 +746,9 @@
         <v/>
       </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>yes</v>
       </c>
     </row>
@@ -751,24 +757,24 @@
         <v>P03</v>
       </c>
       <c r="B3" t="str">
+        <v>Settings</v>
+      </c>
+      <c r="C3" t="str">
         <v>Wake-up time from suspend - YJ(with image)</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>wifi OFF, font size= 4; font = Bookerly; line spacing = medium; margins = default</v>
       </c>
-      <c r="D3" t="str" xml:space="preserve">
+      <c r="E3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Register the device to given account. 
  2. Device should be without ads.
  3. Open the book and go to location 418(Bucket image). 
  3. Put the device in screen saver for 2.30 minutes(suspend). 4. Press the power button and start the timer then stop the timer when the book page is settled. 
  5. Repeat the above step for all the 5 iterations.</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>10</v>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
       <c r="G3" t="str">
         <v/>
       </c>
@@ -788,6 +794,9 @@
         <v/>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>yes</v>
       </c>
     </row>
@@ -796,28 +805,28 @@
         <v>P04</v>
       </c>
       <c r="B4" t="str">
+        <v>store</v>
+      </c>
+      <c r="C4" t="str">
         <v>Warm Book Open: Side Panel Docked Open No annotation</v>
       </c>
-      <c r="C4" t="str" xml:space="preserve">
+      <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">Wi-Fi Off, Chapter 7 next page, Side panel Enabled,
 To Enable Side Panel:
 1)  Enable the side panel from KFT in settings if it’s not already enabled in the Shug book.
 2) Tap on the side panel icon (top right corner) to open the side panel.
 3) Ensure the side panel is docked as it doesn’t overlap the book page.</v>
       </c>
-      <c r="D4" t="str" xml:space="preserve">
+      <c r="E4" t="str" xml:space="preserve">
         <v xml:space="preserve">Step 1: Download and open the Shug book.
 Step 2: Ensure all prerequisites and setups are complete.
 Step 3: Start measuring the time when tapping the (via EPDC logs).
 Step 4: Stop the measurement when the page settles with side panel( Chapter 7, next page).
 Step 5: Repeat Steps 3 and 4 for the next 5 iterations.</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>10</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
       <c r="G4" t="str">
         <v/>
       </c>
@@ -837,6 +846,9 @@
         <v/>
       </c>
       <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
         <v>no</v>
       </c>
     </row>
@@ -845,25 +857,25 @@
         <v>P05</v>
       </c>
       <c r="B5" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C5" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E5" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F5" t="str">
         <v>10</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
       <c r="G5" t="str">
         <v/>
       </c>
@@ -883,6 +895,9 @@
         <v/>
       </c>
       <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
         <v>no</v>
       </c>
     </row>
@@ -891,25 +906,25 @@
         <v>P06</v>
       </c>
       <c r="B6" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C6" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E6" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F6" t="str">
         <v>11</v>
       </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
       <c r="G6" t="str">
         <v/>
       </c>
@@ -929,6 +944,9 @@
         <v/>
       </c>
       <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
         <v>yes</v>
       </c>
     </row>
@@ -937,25 +955,25 @@
         <v>P07</v>
       </c>
       <c r="B7" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C7" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E7" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F7" t="str">
         <v>12</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
       <c r="G7" t="str">
         <v/>
       </c>
@@ -975,6 +993,9 @@
         <v/>
       </c>
       <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
         <v/>
       </c>
     </row>
@@ -983,25 +1004,25 @@
         <v>P08</v>
       </c>
       <c r="B8" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C8" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E8" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F8" t="str">
         <v>13</v>
       </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
       <c r="G8" t="str">
         <v/>
       </c>
@@ -1021,6 +1042,9 @@
         <v/>
       </c>
       <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
         <v/>
       </c>
     </row>
@@ -1029,25 +1053,25 @@
         <v>P09</v>
       </c>
       <c r="B9" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C9" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E9" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F9" t="str">
         <v>14</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
       <c r="G9" t="str">
         <v/>
       </c>
@@ -1067,6 +1091,9 @@
         <v/>
       </c>
       <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
         <v/>
       </c>
     </row>
@@ -1075,25 +1102,25 @@
         <v>P10</v>
       </c>
       <c r="B10" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C10" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E10" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F10" t="str">
         <v>15</v>
       </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
       <c r="G10" t="str">
         <v/>
       </c>
@@ -1113,6 +1140,9 @@
         <v/>
       </c>
       <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
         <v/>
       </c>
     </row>
@@ -1121,25 +1151,25 @@
         <v>P11</v>
       </c>
       <c r="B11" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+        <v>ODAC</v>
       </c>
       <c r="C11" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E11" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F11" t="str">
         <v>16</v>
       </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
       <c r="G11" t="str">
         <v/>
       </c>
@@ -1159,6 +1189,9 @@
         <v/>
       </c>
       <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
         <v/>
       </c>
     </row>
@@ -1166,26 +1199,23 @@
       <c r="A12" t="str">
         <v>P12</v>
       </c>
-      <c r="B12" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C12" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E12" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F12" t="str">
         <v>17</v>
       </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
       <c r="G12" t="str">
         <v/>
       </c>
@@ -1205,6 +1235,9 @@
         <v/>
       </c>
       <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
         <v/>
       </c>
     </row>
@@ -1212,26 +1245,23 @@
       <c r="A13" t="str">
         <v>P13</v>
       </c>
-      <c r="B13" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C13" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D13" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E13" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F13" t="str">
         <v>18</v>
       </c>
-      <c r="F13" t="str">
-        <v/>
-      </c>
       <c r="G13" t="str">
         <v/>
       </c>
@@ -1251,6 +1281,9 @@
         <v/>
       </c>
       <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
         <v/>
       </c>
     </row>
@@ -1258,26 +1291,23 @@
       <c r="A14" t="str">
         <v>P14</v>
       </c>
-      <c r="B14" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C14" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D14" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E14" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F14" t="str">
         <v>19</v>
       </c>
-      <c r="F14" t="str">
-        <v/>
-      </c>
       <c r="G14" t="str">
         <v/>
       </c>
@@ -1297,6 +1327,9 @@
         <v/>
       </c>
       <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
         <v/>
       </c>
     </row>
@@ -1304,26 +1337,23 @@
       <c r="A15" t="str">
         <v>P15</v>
       </c>
-      <c r="B15" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C15" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E15" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F15" t="str">
         <v>20</v>
       </c>
-      <c r="F15" t="str">
-        <v/>
-      </c>
       <c r="G15" t="str">
         <v/>
       </c>
@@ -1343,6 +1373,9 @@
         <v/>
       </c>
       <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
         <v/>
       </c>
     </row>
@@ -1350,26 +1383,23 @@
       <c r="A16" t="str">
         <v>P16</v>
       </c>
-      <c r="B16" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C16" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E16" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F16" t="str">
         <v>21</v>
       </c>
-      <c r="F16" t="str">
-        <v/>
-      </c>
       <c r="G16" t="str">
         <v/>
       </c>
@@ -1389,6 +1419,9 @@
         <v/>
       </c>
       <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
         <v/>
       </c>
     </row>
@@ -1396,26 +1429,23 @@
       <c r="A17" t="str">
         <v>P17</v>
       </c>
-      <c r="B17" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C17" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E17" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F17" t="str">
         <v>22</v>
       </c>
-      <c r="F17" t="str">
-        <v/>
-      </c>
       <c r="G17" t="str">
         <v/>
       </c>
@@ -1435,6 +1465,9 @@
         <v/>
       </c>
       <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
         <v/>
       </c>
     </row>
@@ -1442,26 +1475,23 @@
       <c r="A18" t="str">
         <v>P18</v>
       </c>
-      <c r="B18" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C18" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E18" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F18" t="str">
         <v>23</v>
       </c>
-      <c r="F18" t="str">
-        <v/>
-      </c>
       <c r="G18" t="str">
         <v/>
       </c>
@@ -1481,6 +1511,9 @@
         <v/>
       </c>
       <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
         <v/>
       </c>
     </row>
@@ -1488,26 +1521,23 @@
       <c r="A19" t="str">
         <v>P19</v>
       </c>
-      <c r="B19" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C19" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D19" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E19" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F19" t="str">
         <v>24</v>
       </c>
-      <c r="F19" t="str">
-        <v/>
-      </c>
       <c r="G19" t="str">
         <v/>
       </c>
@@ -1527,6 +1557,9 @@
         <v/>
       </c>
       <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
         <v/>
       </c>
     </row>
@@ -1534,26 +1567,23 @@
       <c r="A20" t="str">
         <v>P20</v>
       </c>
-      <c r="B20" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C20" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D20" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E20" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F20" t="str">
         <v>25</v>
       </c>
-      <c r="F20" t="str">
-        <v/>
-      </c>
       <c r="G20" t="str">
         <v/>
       </c>
@@ -1573,6 +1603,9 @@
         <v/>
       </c>
       <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
         <v/>
       </c>
     </row>
@@ -1580,26 +1613,23 @@
       <c r="A21" t="str">
         <v>P21</v>
       </c>
-      <c r="B21" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C21" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D21" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E21" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F21" t="str">
         <v>26</v>
       </c>
-      <c r="F21" t="str">
-        <v/>
-      </c>
       <c r="G21" t="str">
         <v/>
       </c>
@@ -1619,6 +1649,9 @@
         <v/>
       </c>
       <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
         <v/>
       </c>
     </row>
@@ -1626,26 +1659,23 @@
       <c r="A22" t="str">
         <v>P22</v>
       </c>
-      <c r="B22" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C22" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E22" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F22" t="str">
         <v>27</v>
       </c>
-      <c r="F22" t="str">
-        <v/>
-      </c>
       <c r="G22" t="str">
         <v/>
       </c>
@@ -1665,6 +1695,9 @@
         <v/>
       </c>
       <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
         <v/>
       </c>
     </row>
@@ -1672,26 +1705,23 @@
       <c r="A23" t="str">
         <v>P23</v>
       </c>
-      <c r="B23" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C23" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D23" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E23" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F23" t="str">
         <v>28</v>
       </c>
-      <c r="F23" t="str">
-        <v/>
-      </c>
       <c r="G23" t="str">
         <v/>
       </c>
@@ -1711,6 +1741,9 @@
         <v/>
       </c>
       <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
         <v/>
       </c>
     </row>
@@ -1718,26 +1751,23 @@
       <c r="A24" t="str">
         <v>P24</v>
       </c>
-      <c r="B24" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C24" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E24" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F24" t="str">
         <v>29</v>
       </c>
-      <c r="F24" t="str">
-        <v/>
-      </c>
       <c r="G24" t="str">
         <v/>
       </c>
@@ -1757,6 +1787,9 @@
         <v/>
       </c>
       <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
         <v/>
       </c>
     </row>
@@ -1764,26 +1797,23 @@
       <c r="A25" t="str">
         <v>P25</v>
       </c>
-      <c r="B25" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C25" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E25" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F25" t="str">
         <v>30</v>
       </c>
-      <c r="F25" t="str">
-        <v/>
-      </c>
       <c r="G25" t="str">
         <v/>
       </c>
@@ -1803,6 +1833,9 @@
         <v/>
       </c>
       <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
         <v/>
       </c>
     </row>
@@ -1810,26 +1843,23 @@
       <c r="A26" t="str">
         <v>P26</v>
       </c>
-      <c r="B26" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C26" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D26" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E26" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F26" t="str">
         <v>31</v>
       </c>
-      <c r="F26" t="str">
-        <v/>
-      </c>
       <c r="G26" t="str">
         <v/>
       </c>
@@ -1849,6 +1879,9 @@
         <v/>
       </c>
       <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
         <v/>
       </c>
     </row>
@@ -1856,26 +1889,23 @@
       <c r="A27" t="str">
         <v>P27</v>
       </c>
-      <c r="B27" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C27" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E27" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F27" t="str">
         <v>32</v>
       </c>
-      <c r="F27" t="str">
-        <v/>
-      </c>
       <c r="G27" t="str">
         <v/>
       </c>
@@ -1895,6 +1925,9 @@
         <v/>
       </c>
       <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
         <v/>
       </c>
     </row>
@@ -1902,26 +1935,23 @@
       <c r="A28" t="str">
         <v>P28</v>
       </c>
-      <c r="B28" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C28" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E28" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F28" t="str">
         <v>33</v>
       </c>
-      <c r="F28" t="str">
-        <v/>
-      </c>
       <c r="G28" t="str">
         <v/>
       </c>
@@ -1941,6 +1971,9 @@
         <v/>
       </c>
       <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
         <v/>
       </c>
     </row>
@@ -1948,26 +1981,23 @@
       <c r="A29" t="str">
         <v>P29</v>
       </c>
-      <c r="B29" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C29" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E29" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F29" t="str">
         <v>34</v>
       </c>
-      <c r="F29" t="str">
-        <v/>
-      </c>
       <c r="G29" t="str">
         <v/>
       </c>
@@ -1987,6 +2017,9 @@
         <v/>
       </c>
       <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
         <v/>
       </c>
     </row>
@@ -1994,26 +2027,23 @@
       <c r="A30" t="str">
         <v>P30</v>
       </c>
-      <c r="B30" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C30" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E30" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F30" t="str">
         <v>35</v>
       </c>
-      <c r="F30" t="str">
-        <v/>
-      </c>
       <c r="G30" t="str">
         <v/>
       </c>
@@ -2033,6 +2063,9 @@
         <v/>
       </c>
       <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
         <v/>
       </c>
     </row>
@@ -2040,26 +2073,23 @@
       <c r="A31" t="str">
         <v>P31</v>
       </c>
-      <c r="B31" t="str">
-        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
-      </c>
       <c r="C31" t="str">
-        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
-      </c>
-      <c r="D31" t="str" xml:space="preserve">
-        <v xml:space="preserve">Step 1: Download and open the Shug book.
-Step 2: Ensure all prerequisites and setups are complete.
-Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
-Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
-Step 5: Close the Shug book and re-download it.
-Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
-      </c>
-      <c r="E31" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Step 1: Download and open the Shug book.
+Step 2: Ensure all prerequisites and setups are complete.
+Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).
+Step 4: Stop the measurement when the page settles ( Chapter 7, next page).
+Step 5: Close the Shug book and re-download it.
+Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="F31" t="str">
         <v>36</v>
       </c>
-      <c r="F31" t="str">
-        <v/>
-      </c>
       <c r="G31" t="str">
         <v/>
       </c>
@@ -2079,19 +2109,22 @@
         <v/>
       </c>
       <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N31"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2134,9 +2167,234 @@
         <v>Baseline</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>P05</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ODAC</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Step 1: Download and open the Shug book.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Step 2: Ensure all prerequisites and setups are complete.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Step 4: Stop the measurement when the page settles ( Chapter 7, next page).</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Step 5: Close the Shug book and re-download it.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="B7" t="str">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>P06</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ODAC</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Step 1: Download and open the Shug book.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Step 2: Ensure all prerequisites and setups are complete.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Step 4: Stop the measurement when the page settles ( Chapter 7, next page).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Step 5: Close the Shug book and re-download it.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="B13" t="str">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>P07</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ODAC</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Step 1: Download and open the Shug book.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Step 2: Ensure all prerequisites and setups are complete.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Step 4: Stop the measurement when the page settles ( Chapter 7, next page).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Step 5: Close the Shug book and re-download it.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="B19" t="str">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>P08</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ODAC</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Step 1: Download and open the Shug book.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Step 2: Ensure all prerequisites and setups are complete.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Step 4: Stop the measurement when the page settles ( Chapter 7, next page).</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Step 5: Close the Shug book and re-download it.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="B25" t="str">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>P09</v>
+      </c>
+      <c r="B26" t="str">
+        <v>ODAC</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Warm Book Open: Side Panel Closed - No Annotations</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Wi-Fi Off, Chapter 7 next page, Side panel Disabled</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Step 1: Download and open the Shug book.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Step 2: Ensure all prerequisites and setups are complete.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Step 3: Start measuring the time when tapping the Shug book in the library (via EPDC logs).</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Step 4: Stop the measurement when the page settles ( Chapter 7, next page).</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Step 5: Close the Shug book and re-download it.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Step 6: Repeat Steps 3 to 5 for the next 5 iterations.</v>
+      </c>
+      <c r="B31" t="str">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>